<commit_message>
plantilla para actividades modificada
</commit_message>
<xml_diff>
--- a/assets/templates/plantilla_importacion.xlsx
+++ b/assets/templates/plantilla_importacion.xlsx
@@ -8,7 +8,6 @@
   </bookViews>
   <sheets>
     <sheet name="Actividades" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Instrucciones" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -18,7 +17,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="6">
+  <fonts count="3">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -28,53 +27,21 @@
     </font>
     <font>
       <b val="1"/>
-      <color rgb="FFFFFFFF"/>
-      <sz val="11"/>
-    </font>
-    <font>
-      <i val="1"/>
-      <color rgb="FF888888"/>
-      <sz val="9"/>
+      <sz val="14"/>
     </font>
     <font>
       <b val="1"/>
-      <color rgb="FFFFFFFF"/>
-      <sz val="14"/>
-    </font>
-    <font>
-      <color rgb="FF222222"/>
-      <sz val="10"/>
-    </font>
-    <font>
-      <b val="1"/>
-      <color rgb="FFAA0000"/>
-      <sz val="10"/>
     </font>
   </fonts>
-  <fills count="5">
+  <fills count="2">
     <fill>
       <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
     </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FF0F3460"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFF0F0F0"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFEAF4FB"/>
-      </patternFill>
-    </fill>
   </fills>
-  <borders count="2">
+  <borders count="1">
     <border>
       <left/>
       <right/>
@@ -82,43 +49,20 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin">
-        <color rgb="FFAAAAAA"/>
-      </left>
-      <right style="thin">
-        <color rgb="FFAAAAAA"/>
-      </right>
-      <top style="thin">
-        <color rgb="FFAAAAAA"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="FFAAAAAA"/>
-      </bottom>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -485,213 +429,170 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G3"/>
+  <dimension ref="A1:T3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="28" customWidth="1" min="1" max="1"/>
-    <col width="32" customWidth="1" min="2" max="2"/>
-    <col width="22" customWidth="1" min="3" max="3"/>
-    <col width="22" customWidth="1" min="4" max="4"/>
-    <col width="38" customWidth="1" min="5" max="5"/>
-    <col width="55" customWidth="1" min="6" max="6"/>
-    <col width="20" customWidth="1" min="7" max="7"/>
+    <col width="26" customWidth="1" min="1" max="1"/>
+    <col width="26" customWidth="1" min="2" max="2"/>
+    <col width="26" customWidth="1" min="3" max="3"/>
+    <col width="26" customWidth="1" min="4" max="4"/>
+    <col width="26" customWidth="1" min="5" max="5"/>
+    <col width="26" customWidth="1" min="6" max="6"/>
+    <col width="26" customWidth="1" min="7" max="7"/>
+    <col width="26" customWidth="1" min="8" max="8"/>
+    <col width="26" customWidth="1" min="9" max="9"/>
+    <col width="26" customWidth="1" min="10" max="10"/>
+    <col width="26" customWidth="1" min="11" max="11"/>
+    <col width="26" customWidth="1" min="12" max="12"/>
+    <col width="26" customWidth="1" min="13" max="13"/>
+    <col width="26" customWidth="1" min="14" max="14"/>
+    <col width="26" customWidth="1" min="15" max="15"/>
+    <col width="26" customWidth="1" min="16" max="16"/>
+    <col width="26" customWidth="1" min="17" max="17"/>
+    <col width="26" customWidth="1" min="18" max="18"/>
+    <col width="26" customWidth="1" min="19" max="19"/>
+    <col width="26" customWidth="1" min="20" max="20"/>
   </cols>
   <sheetData>
     <row r="1" ht="30" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>asic</t>
-        </is>
-      </c>
-      <c r="B1" s="1" t="inlineStr">
-        <is>
-          <t>tipo_actividad</t>
-        </is>
-      </c>
-      <c r="C1" s="1" t="inlineStr">
-        <is>
-          <t>fecha_inicio</t>
-        </is>
-      </c>
-      <c r="D1" s="1" t="inlineStr">
-        <is>
-          <t>fecha_fin</t>
-        </is>
-      </c>
-      <c r="E1" s="1" t="inlineStr">
-        <is>
-          <t>lugar</t>
-        </is>
-      </c>
-      <c r="F1" s="1" t="inlineStr">
-        <is>
-          <t>descripcion</t>
-        </is>
-      </c>
-      <c r="G1" s="1" t="inlineStr">
-        <is>
-          <t>participantes</t>
+          <t>REPORTE DE ACTIVIDADES DESARROLLADAS</t>
         </is>
       </c>
     </row>
-    <row r="2" ht="22" customHeight="1">
+    <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>ASIC (nombre exacto)</t>
+          <t>FECHA</t>
         </is>
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>Tipo de Actividad (nombre exacto)</t>
-        </is>
-      </c>
-      <c r="C2" s="2" t="inlineStr">
-        <is>
-          <t>Fecha Inicio (YYYY-MM-DD)</t>
-        </is>
-      </c>
-      <c r="D2" s="2" t="inlineStr">
-        <is>
-          <t>Fecha Fin (YYYY-MM-DD)</t>
-        </is>
-      </c>
-      <c r="E2" s="2" t="inlineStr">
-        <is>
-          <t>Lugar</t>
-        </is>
-      </c>
-      <c r="F2" s="2" t="inlineStr">
-        <is>
-          <t>Descripcion</t>
-        </is>
-      </c>
-      <c r="G2" s="2" t="inlineStr">
-        <is>
-          <t>Participantes (numero)</t>
+          <t>UBICACIÓN</t>
+        </is>
+      </c>
+      <c r="I2" s="2" t="inlineStr">
+        <is>
+          <t>TIPO DE ACTIVIDAD</t>
+        </is>
+      </c>
+      <c r="K2" s="2" t="inlineStr">
+        <is>
+          <t>PARTICIPANTES</t>
         </is>
       </c>
     </row>
-    <row r="3" ht="20" customHeight="1">
+    <row r="3">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>ASIC La Concordia</t>
+          <t>FECHA</t>
         </is>
       </c>
       <c r="B3" s="3" t="inlineStr">
         <is>
-          <t>Charla Educativa</t>
+          <t>ESTADO</t>
         </is>
       </c>
       <c r="C3" s="3" t="inlineStr">
         <is>
-          <t>2025-03-10</t>
+          <t>MUNICIPIO</t>
         </is>
       </c>
       <c r="D3" s="3" t="inlineStr">
         <is>
-          <t>2025-03-10</t>
+          <t>PARROQUIA</t>
         </is>
       </c>
       <c r="E3" s="3" t="inlineStr">
         <is>
-          <t>Ambulatorio Tipo II La Concordia</t>
+          <t>ASIC</t>
         </is>
       </c>
       <c r="F3" s="3" t="inlineStr">
         <is>
-          <t>Charla sobre higiene y prevencion de enfermedades.</t>
+          <t>ESTABLECIMIENTO DE SALUD</t>
         </is>
       </c>
       <c r="G3" s="3" t="inlineStr">
         <is>
-          <t>45</t>
+          <t>NOMBRE DEL ESTABLECIMIENTO DE SALUD</t>
+        </is>
+      </c>
+      <c r="H3" s="3" t="inlineStr">
+        <is>
+          <t>COMITES DE SALUD</t>
+        </is>
+      </c>
+      <c r="I3" s="3" t="inlineStr">
+        <is>
+          <t>ACTIVIDAD DESARROLLADA</t>
+        </is>
+      </c>
+      <c r="J3" s="3" t="inlineStr">
+        <is>
+          <t>TEMA TRATADO</t>
+        </is>
+      </c>
+      <c r="K3" s="3" t="inlineStr">
+        <is>
+          <t>MEDICOS</t>
+        </is>
+      </c>
+      <c r="L3" s="3" t="inlineStr">
+        <is>
+          <t>PROMOTORES EN SALUD</t>
+        </is>
+      </c>
+      <c r="M3" s="3" t="inlineStr">
+        <is>
+          <t>VOCEROS DE COMITÉ DE SALUD</t>
+        </is>
+      </c>
+      <c r="N3" s="3" t="inlineStr">
+        <is>
+          <t>VOCERO DEL CONSEJO DE DIRECCION DEL ASIC</t>
+        </is>
+      </c>
+      <c r="O3" s="3" t="inlineStr">
+        <is>
+          <t>COORDINADOR DE DOCENCIA E INVESTIGACION DEL ASIC</t>
+        </is>
+      </c>
+      <c r="P3" s="3" t="inlineStr">
+        <is>
+          <t>AUTORIDADES PRESENTES</t>
+        </is>
+      </c>
+      <c r="Q3" s="3" t="inlineStr">
+        <is>
+          <t>OTROS ACTORES INVOLUCRADOS</t>
+        </is>
+      </c>
+      <c r="R3" s="3" t="inlineStr">
+        <is>
+          <t>CANTIDAD DE PERSONAS DE LA COMUNIDAD</t>
+        </is>
+      </c>
+      <c r="S3" s="3" t="inlineStr">
+        <is>
+          <t>ESTUDIANTES ASPIRANTES PARA LA SALUD INVOLUCRADOS EN LA ACTIVIDAD</t>
+        </is>
+      </c>
+      <c r="T3" s="3" t="inlineStr">
+        <is>
+          <t>TOTAL DE ASISTENCIA</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:A10"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="80" customWidth="1" min="1" max="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" ht="22" customHeight="1">
-      <c r="A1" s="4" t="inlineStr">
-        <is>
-          <t>INSTRUCCIONES DE USO</t>
-        </is>
-      </c>
-    </row>
-    <row r="2" ht="22" customHeight="1">
-      <c r="A2" s="5" t="inlineStr"/>
-    </row>
-    <row r="3" ht="22" customHeight="1">
-      <c r="A3" s="5" t="inlineStr">
-        <is>
-          <t>1. No modificar los nombres de las columnas de la primera fila (cabecera).</t>
-        </is>
-      </c>
-    </row>
-    <row r="4" ht="22" customHeight="1">
-      <c r="A4" s="5" t="inlineStr">
-        <is>
-          <t>2. La fila 2 es descriptiva (gris claro). Puedes borrarla si lo deseas.</t>
-        </is>
-      </c>
-    </row>
-    <row r="5" ht="22" customHeight="1">
-      <c r="A5" s="6" t="inlineStr">
-        <is>
-          <t>3. La fila 3 es un EJEMPLO. Borrarla antes de importar.</t>
-        </is>
-      </c>
-    </row>
-    <row r="6" ht="22" customHeight="1">
-      <c r="A6" s="5" t="inlineStr">
-        <is>
-          <t>4. El campo ASIC debe coincidir exactamente con el nombre registrado en el sistema.</t>
-        </is>
-      </c>
-    </row>
-    <row r="7" ht="22" customHeight="1">
-      <c r="A7" s="5" t="inlineStr">
-        <is>
-          <t>5. El campo Tipo de Actividad debe coincidir exactamente con el nombre registrado.</t>
-        </is>
-      </c>
-    </row>
-    <row r="8" ht="22" customHeight="1">
-      <c r="A8" s="5" t="inlineStr">
-        <is>
-          <t>6. Las fechas pueden escribirse como YYYY-MM-DD o DD/MM/YYYY.</t>
-        </is>
-      </c>
-    </row>
-    <row r="9" ht="22" customHeight="1">
-      <c r="A9" s="5" t="inlineStr">
-        <is>
-          <t>7. Participantes debe ser un numero entero mayor o igual a 0.</t>
-        </is>
-      </c>
-    </row>
-    <row r="10" ht="22" customHeight="1">
-      <c r="A10" s="5" t="inlineStr">
-        <is>
-          <t>8. Filas completamente vacias seran ignoradas automaticamente.</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
+  <mergeCells count="5">
+    <mergeCell ref="A1:T1"/>
+    <mergeCell ref="I2:J2"/>
+    <mergeCell ref="A2"/>
+    <mergeCell ref="B2:H2"/>
+    <mergeCell ref="K2:T2"/>
+  </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
opcion de vocerias agregada al menu
</commit_message>
<xml_diff>
--- a/assets/templates/plantilla_importacion.xlsx
+++ b/assets/templates/plantilla_importacion.xlsx
@@ -17,7 +17,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="3">
+  <fonts count="7">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -32,16 +32,45 @@
     <font>
       <b val="1"/>
     </font>
+    <font>
+      <sz val="10"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="14"/>
+    </font>
+    <font>
+      <color rgb="00000000"/>
+      <sz val="10"/>
+    </font>
   </fonts>
-  <fills count="2">
+  <fills count="4">
     <fill>
       <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00c00000"/>
+        <bgColor rgb="00c00000"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00e8e8e8"/>
+        <bgColor rgb="00e8e8e8"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="1">
+  <borders count="18">
     <border>
       <left/>
       <right/>
@@ -49,11 +78,199 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin"/>
+      <right style="thin"/>
+      <top style="thin"/>
+      <bottom style="thin"/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="00FFFFFF"/>
+      </left>
+      <right style="thin">
+        <color rgb="00FFFFFF"/>
+      </right>
+      <top style="thin">
+        <color rgb="00FFFFFF"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00FFFFFF"/>
+      </bottom>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color rgb="00FFFFFF"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="00FFFFFF"/>
+      </right>
+      <top style="thin">
+        <color rgb="00FFFFFF"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color rgb="00FFFFFF"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00FFFFFF"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="00FFFFFF"/>
+      </right>
+      <top style="thin">
+        <color rgb="00FFFFFF"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00FFFFFF"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="00FFFFFF"/>
+      </left>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="00FFFFFF"/>
+      </left>
+      <right style="thin">
+        <color rgb="00FFFFFF"/>
+      </right>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="00FFFFFF"/>
+      </left>
+      <right style="thin">
+        <color rgb="00FFFFFF"/>
+      </right>
+      <top/>
+      <bottom style="thin">
+        <color rgb="00FFFFFF"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="00c00000"/>
+      </left>
+      <right style="thin">
+        <color rgb="00c00000"/>
+      </right>
+      <top style="thin">
+        <color rgb="00c00000"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00c00000"/>
+      </bottom>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color rgb="00c00000"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="00c00000"/>
+      </right>
+      <top style="thin">
+        <color rgb="00c00000"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color rgb="00c00000"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00c00000"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="00c00000"/>
+      </right>
+      <top style="thin">
+        <color rgb="00c00000"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00c00000"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="00c00000"/>
+      </left>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="00c00000"/>
+      </left>
+      <right style="thin">
+        <color rgb="00c00000"/>
+      </right>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="00c00000"/>
+      </left>
+      <right style="thin">
+        <color rgb="00c00000"/>
+      </right>
+      <top/>
+      <bottom style="thin">
+        <color rgb="00c00000"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="17">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -62,6 +279,33 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="10" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="10" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="10" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="10" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="13" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="14" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="10" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -138,6 +382,35 @@
     </indexedColors>
   </colors>
 </styleSheet>
+</file>
+
+<file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="TablaImportacion" displayName="TablaImportacion" ref="A3:T4" headerRowCount="1">
+  <autoFilter ref="A3:T4"/>
+  <tableColumns count="20">
+    <tableColumn id="1" name="FECHA"/>
+    <tableColumn id="2" name="ESTADO"/>
+    <tableColumn id="3" name="MUNICIPIO"/>
+    <tableColumn id="4" name="PARROQUIA"/>
+    <tableColumn id="5" name="ASIC"/>
+    <tableColumn id="6" name="ESTABLECIMIENTO DE SALUD ( CDI, SRI, HOSPITAL, CAT, CLINICA POPULAR )"/>
+    <tableColumn id="7" name="NOMBRE DEL ESTABLECIMIENTO DE SALUD"/>
+    <tableColumn id="8" name="COMITES DE SALUD"/>
+    <tableColumn id="9" name="ACTIVIDAD DESARROLLADA"/>
+    <tableColumn id="10" name="TEMA TRATADO"/>
+    <tableColumn id="11" name="MEDICOS"/>
+    <tableColumn id="12" name="PROMOTORES EN SALUD"/>
+    <tableColumn id="13" name="VOCEROS DE COMITE DE SALUD"/>
+    <tableColumn id="14" name="VOCERO DEL CONSEJO DE DIRECCION DEL ASIC"/>
+    <tableColumn id="15" name="COORDINADOR DE DOCENCIA E INVESTIGACION DEL ASIC"/>
+    <tableColumn id="16" name="AUTORIDADES PRESENTES"/>
+    <tableColumn id="17" name="OTROS ACTORES INVOLUCRADOS"/>
+    <tableColumn id="18" name="CANTIDAD DE PERSONAS DE LA COMUNIDAD ( ESTUDIANTES, NIÑOS Y ADULTOS )"/>
+    <tableColumn id="19" name="ESTUDIANTES ASPIRANTES PARA LA SALUD INVOLUCRADOS EN LA ACTIVIDAD"/>
+    <tableColumn id="20" name="TOTAL DE ASISTENCIA"/>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleMedium9" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</table>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -429,7 +702,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:T3"/>
+  <dimension ref="A1:T4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
@@ -452,147 +725,210 @@
     <col width="26" customWidth="1" min="18" max="18"/>
     <col width="26" customWidth="1" min="19" max="19"/>
     <col width="26" customWidth="1" min="20" max="20"/>
+    <col hidden="1" outlineLevel="1" width="13" customWidth="1" min="21" max="16384"/>
   </cols>
   <sheetData>
     <row r="1" ht="30" customHeight="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" s="13" t="inlineStr">
         <is>
           <t>REPORTE DE ACTIVIDADES DESARROLLADAS</t>
         </is>
       </c>
+      <c r="B1" s="13" t="n"/>
+      <c r="C1" s="13" t="n"/>
+      <c r="D1" s="13" t="n"/>
+      <c r="E1" s="13" t="n"/>
+      <c r="F1" s="13" t="n"/>
+      <c r="G1" s="13" t="n"/>
+      <c r="H1" s="13" t="n"/>
+      <c r="I1" s="13" t="n"/>
+      <c r="J1" s="13" t="n"/>
+      <c r="K1" s="13" t="n"/>
+      <c r="L1" s="13" t="n"/>
+      <c r="M1" s="13" t="n"/>
+      <c r="N1" s="13" t="n"/>
+      <c r="O1" s="13" t="n"/>
+      <c r="P1" s="13" t="n"/>
+      <c r="Q1" s="13" t="n"/>
+      <c r="R1" s="13" t="n"/>
+      <c r="S1" s="13" t="n"/>
+      <c r="T1" s="13" t="n"/>
     </row>
     <row r="2">
-      <c r="A2" s="2" t="inlineStr">
+      <c r="A2" s="16" t="inlineStr">
         <is>
           <t>FECHA</t>
         </is>
       </c>
-      <c r="B2" s="2" t="inlineStr">
+      <c r="B2" s="16" t="inlineStr">
         <is>
           <t>UBICACIÓN</t>
         </is>
       </c>
-      <c r="I2" s="2" t="inlineStr">
+      <c r="C2" s="16" t="n"/>
+      <c r="D2" s="16" t="n"/>
+      <c r="E2" s="16" t="n"/>
+      <c r="F2" s="16" t="n"/>
+      <c r="G2" s="16" t="n"/>
+      <c r="H2" s="16" t="n"/>
+      <c r="I2" s="16" t="inlineStr">
         <is>
           <t>TIPO DE ACTIVIDAD</t>
         </is>
       </c>
-      <c r="K2" s="2" t="inlineStr">
+      <c r="J2" s="16" t="n"/>
+      <c r="K2" s="16" t="inlineStr">
         <is>
           <t>PARTICIPANTES</t>
         </is>
       </c>
+      <c r="L2" s="16" t="n"/>
+      <c r="M2" s="16" t="n"/>
+      <c r="N2" s="16" t="n"/>
+      <c r="O2" s="16" t="n"/>
+      <c r="P2" s="16" t="n"/>
+      <c r="Q2" s="16" t="n"/>
+      <c r="R2" s="16" t="n"/>
+      <c r="S2" s="16" t="n"/>
+      <c r="T2" s="16" t="n"/>
     </row>
     <row r="3">
-      <c r="A3" s="3" t="inlineStr">
+      <c r="A3" s="16" t="inlineStr">
         <is>
           <t>FECHA</t>
         </is>
       </c>
-      <c r="B3" s="3" t="inlineStr">
+      <c r="B3" s="16" t="inlineStr">
         <is>
           <t>ESTADO</t>
         </is>
       </c>
-      <c r="C3" s="3" t="inlineStr">
+      <c r="C3" s="16" t="inlineStr">
         <is>
           <t>MUNICIPIO</t>
         </is>
       </c>
-      <c r="D3" s="3" t="inlineStr">
+      <c r="D3" s="16" t="inlineStr">
         <is>
           <t>PARROQUIA</t>
         </is>
       </c>
-      <c r="E3" s="3" t="inlineStr">
+      <c r="E3" s="16" t="inlineStr">
         <is>
           <t>ASIC</t>
         </is>
       </c>
-      <c r="F3" s="3" t="inlineStr">
-        <is>
-          <t>ESTABLECIMIENTO DE SALUD</t>
-        </is>
-      </c>
-      <c r="G3" s="3" t="inlineStr">
+      <c r="F3" s="16" t="inlineStr">
+        <is>
+          <t>ESTABLECIMIENTO DE SALUD ( CDI, SRI, HOSPITAL, CAT, CLINICA POPULAR )</t>
+        </is>
+      </c>
+      <c r="G3" s="16" t="inlineStr">
         <is>
           <t>NOMBRE DEL ESTABLECIMIENTO DE SALUD</t>
         </is>
       </c>
-      <c r="H3" s="3" t="inlineStr">
+      <c r="H3" s="16" t="inlineStr">
         <is>
           <t>COMITES DE SALUD</t>
         </is>
       </c>
-      <c r="I3" s="3" t="inlineStr">
+      <c r="I3" s="16" t="inlineStr">
         <is>
           <t>ACTIVIDAD DESARROLLADA</t>
         </is>
       </c>
-      <c r="J3" s="3" t="inlineStr">
+      <c r="J3" s="16" t="inlineStr">
         <is>
           <t>TEMA TRATADO</t>
         </is>
       </c>
-      <c r="K3" s="3" t="inlineStr">
+      <c r="K3" s="16" t="inlineStr">
         <is>
           <t>MEDICOS</t>
         </is>
       </c>
-      <c r="L3" s="3" t="inlineStr">
+      <c r="L3" s="16" t="inlineStr">
         <is>
           <t>PROMOTORES EN SALUD</t>
         </is>
       </c>
-      <c r="M3" s="3" t="inlineStr">
-        <is>
-          <t>VOCEROS DE COMITÉ DE SALUD</t>
-        </is>
-      </c>
-      <c r="N3" s="3" t="inlineStr">
+      <c r="M3" s="16" t="inlineStr">
+        <is>
+          <t>VOCEROS DE COMITE DE SALUD</t>
+        </is>
+      </c>
+      <c r="N3" s="16" t="inlineStr">
         <is>
           <t>VOCERO DEL CONSEJO DE DIRECCION DEL ASIC</t>
         </is>
       </c>
-      <c r="O3" s="3" t="inlineStr">
+      <c r="O3" s="16" t="inlineStr">
         <is>
           <t>COORDINADOR DE DOCENCIA E INVESTIGACION DEL ASIC</t>
         </is>
       </c>
-      <c r="P3" s="3" t="inlineStr">
+      <c r="P3" s="16" t="inlineStr">
         <is>
           <t>AUTORIDADES PRESENTES</t>
         </is>
       </c>
-      <c r="Q3" s="3" t="inlineStr">
+      <c r="Q3" s="16" t="inlineStr">
         <is>
           <t>OTROS ACTORES INVOLUCRADOS</t>
         </is>
       </c>
-      <c r="R3" s="3" t="inlineStr">
-        <is>
-          <t>CANTIDAD DE PERSONAS DE LA COMUNIDAD</t>
-        </is>
-      </c>
-      <c r="S3" s="3" t="inlineStr">
+      <c r="R3" s="16" t="inlineStr">
+        <is>
+          <t>CANTIDAD DE PERSONAS DE LA COMUNIDAD ( ESTUDIANTES, NIÑOS Y ADULTOS )</t>
+        </is>
+      </c>
+      <c r="S3" s="16" t="inlineStr">
         <is>
           <t>ESTUDIANTES ASPIRANTES PARA LA SALUD INVOLUCRADOS EN LA ACTIVIDAD</t>
         </is>
       </c>
-      <c r="T3" s="3" t="inlineStr">
+      <c r="T3" s="16" t="inlineStr">
         <is>
           <t>TOTAL DE ASISTENCIA</t>
         </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="12" t="n"/>
+      <c r="B4" s="12" t="n"/>
+      <c r="C4" s="12" t="n"/>
+      <c r="D4" s="12" t="n"/>
+      <c r="E4" s="12" t="n"/>
+      <c r="F4" s="12" t="n"/>
+      <c r="G4" s="12" t="n"/>
+      <c r="H4" s="12" t="n"/>
+      <c r="I4" s="12" t="n"/>
+      <c r="J4" s="12" t="n"/>
+      <c r="K4" s="12" t="n"/>
+      <c r="L4" s="12" t="n"/>
+      <c r="M4" s="12" t="n"/>
+      <c r="N4" s="12" t="n"/>
+      <c r="O4" s="12" t="n"/>
+      <c r="P4" s="12" t="n"/>
+      <c r="Q4" s="12" t="n"/>
+      <c r="R4" s="12" t="n"/>
+      <c r="S4" s="12" t="n"/>
+      <c r="T4" s="12">
+        <f>IF(COUNTA(K4:S4)&gt;0,SUM(K4:S4),"")</f>
+        <v/>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="5">
+  <mergeCells count="4">
     <mergeCell ref="A1:T1"/>
     <mergeCell ref="I2:J2"/>
-    <mergeCell ref="A2"/>
     <mergeCell ref="B2:H2"/>
     <mergeCell ref="K2:T2"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <tableParts count="1">
+    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+  </tableParts>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
ajustes y mejoras en la plantilla excel
</commit_message>
<xml_diff>
--- a/assets/templates/plantilla_importacion.xlsx
+++ b/assets/templates/plantilla_importacion.xlsx
@@ -16,7 +16,9 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="0"/>
+  <numFmts count="1">
+    <numFmt numFmtId="164" formatCode="m/d/yyyy"/>
+  </numFmts>
   <fonts count="7">
     <font>
       <name val="Calibri"/>
@@ -270,7 +272,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="17">
+  <cellXfs count="19">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -306,6 +308,10 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="13" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="14" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="2" borderId="10" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="6" fillId="3" borderId="10" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -705,7 +711,7 @@
   <dimension ref="A1:T4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="26" customWidth="1" min="1" max="1"/>
+    <col width="26" customWidth="1" style="17" min="1" max="1"/>
     <col width="26" customWidth="1" min="2" max="2"/>
     <col width="26" customWidth="1" min="3" max="3"/>
     <col width="26" customWidth="1" min="4" max="4"/>
@@ -734,25 +740,25 @@
           <t>REPORTE DE ACTIVIDADES DESARROLLADAS</t>
         </is>
       </c>
-      <c r="B1" s="13" t="n"/>
-      <c r="C1" s="13" t="n"/>
-      <c r="D1" s="13" t="n"/>
-      <c r="E1" s="13" t="n"/>
-      <c r="F1" s="13" t="n"/>
-      <c r="G1" s="13" t="n"/>
-      <c r="H1" s="13" t="n"/>
-      <c r="I1" s="13" t="n"/>
-      <c r="J1" s="13" t="n"/>
-      <c r="K1" s="13" t="n"/>
-      <c r="L1" s="13" t="n"/>
-      <c r="M1" s="13" t="n"/>
-      <c r="N1" s="13" t="n"/>
-      <c r="O1" s="13" t="n"/>
-      <c r="P1" s="13" t="n"/>
-      <c r="Q1" s="13" t="n"/>
-      <c r="R1" s="13" t="n"/>
-      <c r="S1" s="13" t="n"/>
-      <c r="T1" s="13" t="n"/>
+      <c r="B1" s="14" t="n"/>
+      <c r="C1" s="14" t="n"/>
+      <c r="D1" s="14" t="n"/>
+      <c r="E1" s="14" t="n"/>
+      <c r="F1" s="14" t="n"/>
+      <c r="G1" s="14" t="n"/>
+      <c r="H1" s="14" t="n"/>
+      <c r="I1" s="14" t="n"/>
+      <c r="J1" s="14" t="n"/>
+      <c r="K1" s="14" t="n"/>
+      <c r="L1" s="14" t="n"/>
+      <c r="M1" s="14" t="n"/>
+      <c r="N1" s="14" t="n"/>
+      <c r="O1" s="14" t="n"/>
+      <c r="P1" s="14" t="n"/>
+      <c r="Q1" s="14" t="n"/>
+      <c r="R1" s="14" t="n"/>
+      <c r="S1" s="14" t="n"/>
+      <c r="T1" s="15" t="n"/>
     </row>
     <row r="2">
       <c r="A2" s="16" t="inlineStr">
@@ -765,32 +771,32 @@
           <t>UBICACIÓN</t>
         </is>
       </c>
-      <c r="C2" s="16" t="n"/>
-      <c r="D2" s="16" t="n"/>
-      <c r="E2" s="16" t="n"/>
-      <c r="F2" s="16" t="n"/>
-      <c r="G2" s="16" t="n"/>
-      <c r="H2" s="16" t="n"/>
+      <c r="C2" s="14" t="n"/>
+      <c r="D2" s="14" t="n"/>
+      <c r="E2" s="14" t="n"/>
+      <c r="F2" s="14" t="n"/>
+      <c r="G2" s="14" t="n"/>
+      <c r="H2" s="15" t="n"/>
       <c r="I2" s="16" t="inlineStr">
         <is>
           <t>TIPO DE ACTIVIDAD</t>
         </is>
       </c>
-      <c r="J2" s="16" t="n"/>
+      <c r="J2" s="15" t="n"/>
       <c r="K2" s="16" t="inlineStr">
         <is>
           <t>PARTICIPANTES</t>
         </is>
       </c>
-      <c r="L2" s="16" t="n"/>
-      <c r="M2" s="16" t="n"/>
-      <c r="N2" s="16" t="n"/>
-      <c r="O2" s="16" t="n"/>
-      <c r="P2" s="16" t="n"/>
-      <c r="Q2" s="16" t="n"/>
-      <c r="R2" s="16" t="n"/>
-      <c r="S2" s="16" t="n"/>
-      <c r="T2" s="16" t="n"/>
+      <c r="L2" s="14" t="n"/>
+      <c r="M2" s="14" t="n"/>
+      <c r="N2" s="14" t="n"/>
+      <c r="O2" s="14" t="n"/>
+      <c r="P2" s="14" t="n"/>
+      <c r="Q2" s="14" t="n"/>
+      <c r="R2" s="14" t="n"/>
+      <c r="S2" s="14" t="n"/>
+      <c r="T2" s="15" t="n"/>
     </row>
     <row r="3">
       <c r="A3" s="16" t="inlineStr">
@@ -895,7 +901,7 @@
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="12" t="n"/>
+      <c r="A4" s="18" t="n"/>
       <c r="B4" s="12" t="n"/>
       <c r="C4" s="12" t="n"/>
       <c r="D4" s="12" t="n"/>
@@ -922,10 +928,25 @@
   </sheetData>
   <mergeCells count="4">
     <mergeCell ref="A1:T1"/>
+    <mergeCell ref="B2:H2"/>
     <mergeCell ref="I2:J2"/>
-    <mergeCell ref="B2:H2"/>
     <mergeCell ref="K2:T2"/>
   </mergeCells>
+  <dataValidations count="4">
+    <dataValidation sqref="B4:B1048576" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Estado no válido" error="Selecciona Táchira." promptTitle="Estado" prompt="Selecciona el estado." type="list">
+      <formula1>"Táchira"</formula1>
+    </dataValidation>
+    <dataValidation sqref="C4:C1048576" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Municipio no válido" error="Selecciona San Cristobal o Ayacucho." promptTitle="Municipio" prompt="Selecciona el municipio." type="list">
+      <formula1>"San Cristobal,Ayacucho"</formula1>
+    </dataValidation>
+    <dataValidation sqref="A4:A1048576" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Fecha no válida" error="Introduce una fecha válida." promptTitle="Fecha" prompt="Selecciona o introduce una fecha." type="date" operator="between">
+      <formula1>DATE(1900,1,1)</formula1>
+      <formula2>DATE(2100,12,31)</formula2>
+    </dataValidation>
+    <dataValidation sqref="I4:I1048576" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Actividad no válida" error="Selecciona una actividad del catálogo." promptTitle="Actividad desarrollada" prompt="Selecciona el tipo de actividad." type="list">
+      <formula1>"Jornada de Vacunación,Consulta Médica,Charla de Salud,Jornada Odontológica,Actividad Deportiva"</formula1>
+    </dataValidation>
+  </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <tableParts count="1">
     <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>

</xml_diff>

<commit_message>
mejoras en la plantilla
</commit_message>
<xml_diff>
--- a/assets/templates/plantilla_importacion.xlsx
+++ b/assets/templates/plantilla_importacion.xlsx
@@ -932,19 +932,22 @@
     <mergeCell ref="I2:J2"/>
     <mergeCell ref="K2:T2"/>
   </mergeCells>
-  <dataValidations count="4">
+  <dataValidations count="5">
     <dataValidation sqref="B4:B1048576" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Estado no válido" error="Selecciona Táchira." promptTitle="Estado" prompt="Selecciona el estado." type="list">
       <formula1>"Táchira"</formula1>
     </dataValidation>
-    <dataValidation sqref="C4:C1048576" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Municipio no válido" error="Selecciona San Cristobal o Ayacucho." promptTitle="Municipio" prompt="Selecciona el municipio." type="list">
-      <formula1>"San Cristobal,Ayacucho"</formula1>
+    <dataValidation sqref="C4:C1048576" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Municipio no válido" error="Selecciona un municipio del catálogo." promptTitle="Municipio" prompt="Selecciona el municipio." type="list">
+      <formula1>"Andrés Bello,Antonio Rómulo Costa,Ayacucho,Bolívar,Capacho Independencia,Capacho Libertad,Cárdenas,Córdoba,Dr. Hugo Murzi,Dr. Jacinto Convit,Dr. José María Vargas,Fernández Feo,García de Hevia,Guásimos,Jáuregui,Junín,Libertador,Michelena,Panamericano,Sabaneta,Samuel Darío Maldonado,Sucre,Torbes,Ureña,Uribante"</formula1>
     </dataValidation>
     <dataValidation sqref="A4:A1048576" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Fecha no válida" error="Introduce una fecha válida." promptTitle="Fecha" prompt="Selecciona o introduce una fecha." type="date" operator="between">
       <formula1>DATE(1900,1,1)</formula1>
       <formula2>DATE(2100,12,31)</formula2>
     </dataValidation>
     <dataValidation sqref="I4:I1048576" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Actividad no válida" error="Selecciona una actividad del catálogo." promptTitle="Actividad desarrollada" prompt="Selecciona el tipo de actividad." type="list">
-      <formula1>"Jornada de Vacunación,Consulta Médica,Charla de Salud,Jornada Odontológica,Actividad Deportiva"</formula1>
+      <formula1>"Salud toca tu puerta,Sesiones educativas,Los Comités de Salud van a la escuela,Actividades de Promoción y Prevención Social,Participación Activa en Jornadas,Participación Activa en Inmunizaciones,Entrevista servicio social"</formula1>
+    </dataValidation>
+    <dataValidation sqref="E4:E1048576" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="ASIC no válido" error="Selecciona un ASIC del catálogo." promptTitle="ASIC" prompt="Selecciona el ASIC." type="list">
+      <formula1>"Andrés Bello,Antonio Rómulo Costa,Ayacucho,Bolívar,Capacho Independencia,Capacho Libertad,Cárdenas,Córdoba,Dr. Hugo Murzi,Dr. Jacinto Convit,Dr. José María Vargas,Fernández Feo,García de Hevia,Guásimos,Jáuregui,Junín,Libertador,Michelena,Panamericano,Sabaneta,Samuel Darío Maldonado,Sucre,Torbes,Ureña,Uribante"</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>